<commit_message>
fix : Inventory Add Item
인벤토리에 아이템을 추가하는 기능 수정
</commit_message>
<xml_diff>
--- a/RPGProject/Assets/Project/Data/ExcelData/ItemInfo.xlsx
+++ b/RPGProject/Assets/Project/Data/ExcelData/ItemInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suyb1\Documents\GitHub\RPG\RPGProject\Assets\Project\Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75AA5B7-1026-4918-BEB0-F237251BCB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D579B145-BA2A-4D57-A520-408BD644A39C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13575" yWindow="2205" windowWidth="14790" windowHeight="10695" xr2:uid="{3510F260-6A7D-4843-A2DA-E1BA315C89A0}"/>
+    <workbookView xWindow="9075" yWindow="3780" windowWidth="14790" windowHeight="10695" xr2:uid="{3510F260-6A7D-4843-A2DA-E1BA315C89A0}"/>
   </bookViews>
   <sheets>
     <sheet name="test" sheetId="1" r:id="rId1"/>

</xml_diff>